<commit_message>
adición de capturas de pantalla
</commit_message>
<xml_diff>
--- a/datos/Registros.xlsx
+++ b/datos/Registros.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="81">
   <si>
     <t>order_id</t>
   </si>
@@ -48,108 +48,108 @@
     <t>total</t>
   </si>
   <si>
-    <t>Daniel64</t>
+    <t>Daniel109</t>
   </si>
   <si>
     <t>Daniel</t>
   </si>
   <si>
+    <t>PROD-005</t>
+  </si>
+  <si>
+    <t>Impresora térmica de etiquetas</t>
+  </si>
+  <si>
+    <t>DESPACHADO</t>
+  </si>
+  <si>
+    <t>precio_unitario</t>
+  </si>
+  <si>
+    <t>PROD-001</t>
+  </si>
+  <si>
+    <t>Caja de guantes industriales talla M</t>
+  </si>
+  <si>
+    <t>PROD-002</t>
+  </si>
+  <si>
+    <t>Cinta de embalaje 48 mm x 100 m</t>
+  </si>
+  <si>
+    <t>PROD-003</t>
+  </si>
+  <si>
+    <t>Rollo de etiqueta térmica 100x100</t>
+  </si>
+  <si>
+    <t>PROD-004</t>
+  </si>
+  <si>
+    <t>Lector de código de barras inalámbrico</t>
+  </si>
+  <si>
+    <t>PROD-006</t>
+  </si>
+  <si>
+    <t>Pallet plástico estándar 120x100 cm</t>
+  </si>
+  <si>
+    <t>PROD-007</t>
+  </si>
+  <si>
+    <t>Chaleco reflectivo de seguridad</t>
+  </si>
+  <si>
+    <t>PROD-008</t>
+  </si>
+  <si>
+    <t>Botas de seguridad punta de acero</t>
+  </si>
+  <si>
+    <t>PROD-009</t>
+  </si>
+  <si>
+    <t>Carretilla de carga plegable</t>
+  </si>
+  <si>
+    <t>PROD-010</t>
+  </si>
+  <si>
+    <t>Escáner handheld para inventario</t>
+  </si>
+  <si>
+    <t>PROD-011</t>
+  </si>
+  <si>
+    <t>Bolsa courier impermeable mediana</t>
+  </si>
+  <si>
+    <t>PROD-012</t>
+  </si>
+  <si>
+    <t>Selladora manual para empaque</t>
+  </si>
+  <si>
+    <t>PROD-013</t>
+  </si>
+  <si>
+    <t>Caja corrugada mediana 40x30x30</t>
+  </si>
+  <si>
+    <t>PROD-014</t>
+  </si>
+  <si>
+    <t>Film stretch industrial 500 m</t>
+  </si>
+  <si>
     <t>PROD-015</t>
   </si>
   <si>
     <t>Tablet rugerizada para reparto</t>
   </si>
   <si>
-    <t>DESPACHADO</t>
-  </si>
-  <si>
-    <t>precio_unitario</t>
-  </si>
-  <si>
-    <t>PROD-001</t>
-  </si>
-  <si>
-    <t>Caja de guantes industriales talla M</t>
-  </si>
-  <si>
-    <t>PROD-002</t>
-  </si>
-  <si>
-    <t>Cinta de embalaje 48 mm x 100 m</t>
-  </si>
-  <si>
-    <t>PROD-003</t>
-  </si>
-  <si>
-    <t>Rollo de etiqueta térmica 100x100</t>
-  </si>
-  <si>
-    <t>PROD-004</t>
-  </si>
-  <si>
-    <t>Lector de código de barras inalámbrico</t>
-  </si>
-  <si>
-    <t>PROD-005</t>
-  </si>
-  <si>
-    <t>Impresora térmica de etiquetas</t>
-  </si>
-  <si>
-    <t>PROD-006</t>
-  </si>
-  <si>
-    <t>Pallet plástico estándar 120x100 cm</t>
-  </si>
-  <si>
-    <t>PROD-007</t>
-  </si>
-  <si>
-    <t>Chaleco reflectivo de seguridad</t>
-  </si>
-  <si>
-    <t>PROD-008</t>
-  </si>
-  <si>
-    <t>Botas de seguridad punta de acero</t>
-  </si>
-  <si>
-    <t>PROD-009</t>
-  </si>
-  <si>
-    <t>Carretilla de carga plegable</t>
-  </si>
-  <si>
-    <t>PROD-010</t>
-  </si>
-  <si>
-    <t>Escáner handheld para inventario</t>
-  </si>
-  <si>
-    <t>PROD-011</t>
-  </si>
-  <si>
-    <t>Bolsa courier impermeable mediana</t>
-  </si>
-  <si>
-    <t>PROD-012</t>
-  </si>
-  <si>
-    <t>Selladora manual para empaque</t>
-  </si>
-  <si>
-    <t>PROD-013</t>
-  </si>
-  <si>
-    <t>Caja corrugada mediana 40x30x30</t>
-  </si>
-  <si>
-    <t>PROD-014</t>
-  </si>
-  <si>
-    <t>Film stretch industrial 500 m</t>
-  </si>
-  <si>
     <t>PROD-016</t>
   </si>
   <si>
@@ -252,31 +252,10 @@
     <t>estado_factura</t>
   </si>
   <si>
-    <t>FAC-</t>
+    <t>FAC-Daniel109</t>
   </si>
   <si>
     <t>GENERADA</t>
-  </si>
-  <si>
-    <t>FAC-Daniel58-58</t>
-  </si>
-  <si>
-    <t>Daniel58-58</t>
-  </si>
-  <si>
-    <t>FAC-Daniel60-60</t>
-  </si>
-  <si>
-    <t>Daniel60-60</t>
-  </si>
-  <si>
-    <t>FAC-Daniel62</t>
-  </si>
-  <si>
-    <t>Daniel62</t>
-  </si>
-  <si>
-    <t>FAC-Daniel64</t>
   </si>
 </sst>
 </file>
@@ -799,16 +778,16 @@
         <v>15</v>
       </c>
       <c r="H2" s="4">
-        <v>5.0</v>
+        <v>6.0</v>
       </c>
       <c r="I2" s="6">
-        <v>46176.64761574074</v>
+        <v>46181.57429398148</v>
       </c>
       <c r="J2" s="6">
-        <v>46176.647673611114</v>
+        <v>46181.57643518518</v>
       </c>
       <c r="K2" s="7">
-        <v>890000.0</v>
+        <v>420000.0</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
@@ -1254,10 +1233,10 @@
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="13" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="C6" s="14">
         <v>6.0</v>
@@ -1268,10 +1247,10 @@
     </row>
     <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="13" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C7" s="14">
         <v>18.0</v>
@@ -1282,10 +1261,10 @@
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="13" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C8" s="14">
         <v>55.0</v>
@@ -1296,10 +1275,10 @@
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="13" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C9" s="14">
         <v>30.0</v>
@@ -1310,10 +1289,10 @@
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="13" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C10" s="14">
         <v>10.0</v>
@@ -1324,10 +1303,10 @@
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C11" s="14">
         <v>8.0</v>
@@ -1338,10 +1317,10 @@
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="13" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C12" s="14">
         <v>200.0</v>
@@ -1352,10 +1331,10 @@
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C13" s="14">
         <v>14.0</v>
@@ -1366,10 +1345,10 @@
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="13" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C14" s="14">
         <v>150.0</v>
@@ -1380,10 +1359,10 @@
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="13" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C15" s="14">
         <v>34.0</v>
@@ -1394,10 +1373,10 @@
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="13" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>14</v>
+        <v>44</v>
       </c>
       <c r="C16" s="14">
         <v>5.0</v>
@@ -1667,129 +1646,69 @@
       <c r="A2" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
+      <c r="B2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>12</v>
+      </c>
       <c r="D2" s="7">
-        <v>96000.0</v>
+        <v>420000.0</v>
       </c>
       <c r="E2" s="16">
-        <v>46176.639375</v>
+        <v>46181.57643518518</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="3" t="s">
-        <v>79</v>
-      </c>
+      <c r="A3" s="3"/>
       <c r="B3" s="10"/>
       <c r="C3" s="10"/>
-      <c r="D3" s="7">
-        <v>14500.0</v>
-      </c>
-      <c r="E3" s="16">
-        <v>46176.640335648146</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>80</v>
-      </c>
+      <c r="D3" s="7"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="5"/>
     </row>
     <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="3" t="s">
-        <v>79</v>
-      </c>
+      <c r="A4" s="3"/>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
-      <c r="D4" s="7">
-        <v>96000.0</v>
-      </c>
-      <c r="E4" s="16">
-        <v>46176.64131944445</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>80</v>
-      </c>
+      <c r="D4" s="7"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="5"/>
     </row>
     <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="7">
-        <v>96000.0</v>
-      </c>
-      <c r="E5" s="16">
-        <v>46176.643900462965</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>80</v>
-      </c>
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="5"/>
     </row>
     <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="7">
-        <v>890000.0</v>
-      </c>
-      <c r="E6" s="16">
-        <v>46176.64480324074</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>80</v>
-      </c>
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="5"/>
     </row>
     <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="7">
-        <v>890000.0</v>
-      </c>
-      <c r="E7" s="16">
-        <v>46176.646631944444</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>80</v>
-      </c>
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="5"/>
     </row>
     <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="7">
-        <v>890000.0</v>
-      </c>
-      <c r="E8" s="16">
-        <v>46176.647673611114</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>80</v>
-      </c>
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="5"/>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="10"/>

</xml_diff>